<commit_message>
feat(flux-klein): add Flux 2 Klein 9B workflow with avatar reference and Day 101 image-only entry
</commit_message>
<xml_diff>
--- a/Zara_Khan_Optimized_Calendar.xlsx
+++ b/Zara_Khan_Optimized_Calendar.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T73"/>
+  <dimension ref="A1:T74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5265,6 +5265,80 @@
         <v>115</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DAY101_POST_01</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Day 101</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Feed Photo</t>
+        </is>
+      </c>
+      <c r="E74" t="b">
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Zara Khan quiet morning aesthetic in sunlit South Mumbai heritage cafe patio reading book with coffee</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Natural warm morning light streaming through vintage wooden blinds, ivory linen button-up shirt, layered delicate gold necklaces, relaxed candid smile, 35mm film aesthetic, Zara Khan avatar reference consistency</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>The quietest hours of Bombay are always the most poetic. Linen mornings and black coffee.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Acoustic lo-fi warm morning guitar chords</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>https://in.pinterest.com/pin/1105985746020500854/</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1IaeGtZF6cLdXTyREF6HiDwyY3x9_0sOf</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>ZARA_KHAN.png</t>
+        </is>
+      </c>
+      <c r="T74" t="n">
+        <v>184</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>